<commit_message>
Actualizacion de CRUDS con copilot
</commit_message>
<xml_diff>
--- a/archivos/tabla_roles.xlsx
+++ b/archivos/tabla_roles.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24026"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70186259-6DC2-4632-A091-1CF3D4790825}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FE167A8-41F6-4C3A-8E1D-165DC2E3FD54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -13,14 +13,14 @@
     <sheet name="Hoja3" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$B$171</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$B$237</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="78">
   <si>
     <t>dir</t>
   </si>
@@ -236,6 +236,24 @@
   </si>
   <si>
     <t>views/tika_siembras_erradicaciones.php</t>
+  </si>
+  <si>
+    <t>views/report_pb_compara_prod.php</t>
+  </si>
+  <si>
+    <t>views/programs.php</t>
+  </si>
+  <si>
+    <t>views/programsf.php</t>
+  </si>
+  <si>
+    <t>views/proyectos.php</t>
+  </si>
+  <si>
+    <t>views/tareas.php</t>
+  </si>
+  <si>
+    <t>views/bitacora.php</t>
   </si>
 </sst>
 </file>
@@ -300,9 +318,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -340,9 +358,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -375,9 +393,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -410,9 +445,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -586,10 +638,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B200"/>
+  <dimension ref="A1:B237"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -890,295 +943,295 @@
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="B38">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="B39">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="B40">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B41">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B42">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B43">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B44">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B45">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B46">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B47">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B48">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B49">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B50">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B51">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B52">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B53">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B54">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B55">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B56">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B57">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B58">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B59">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B60">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B61">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B62">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B63">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B64">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B65">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B66">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B67">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B68">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B69">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B70">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B71">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B72">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B73">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="B74">
         <v>0</v>
@@ -1186,7 +1239,7 @@
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="B75">
         <v>0</v>
@@ -1194,7 +1247,7 @@
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="B76">
         <v>0</v>
@@ -1202,191 +1255,191 @@
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>5</v>
+        <v>38</v>
       </c>
       <c r="B77">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="B78">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>7</v>
+        <v>40</v>
       </c>
       <c r="B79">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>8</v>
-      </c>
-      <c r="B80">
-        <v>0</v>
+        <v>41</v>
+      </c>
+      <c r="B80" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>9</v>
+        <v>42</v>
       </c>
       <c r="B81">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="B82">
-        <v>0</v>
+        <v>19</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="B83">
-        <v>0</v>
+        <v>19</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="B84">
-        <v>0</v>
+        <v>19</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="B85">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B86">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="B87">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="B88">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>17</v>
+        <v>43</v>
       </c>
       <c r="B89">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="B90">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="B91">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="B92">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="B93">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="B94">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="B95">
-        <v>3</v>
+        <v>20</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="B96">
-        <v>3</v>
+        <v>19</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>25</v>
+        <v>52</v>
       </c>
       <c r="B97">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>26</v>
+        <v>47</v>
       </c>
       <c r="B98">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="B99">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>28</v>
+        <v>47</v>
       </c>
       <c r="B100">
         <v>3</v>
@@ -1394,7 +1447,7 @@
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>29</v>
+        <v>48</v>
       </c>
       <c r="B101">
         <v>3</v>
@@ -1402,15 +1455,15 @@
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="B102">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="B103">
         <v>3</v>
@@ -1418,7 +1471,7 @@
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B104">
         <v>3</v>
@@ -1426,79 +1479,79 @@
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="B105">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>34</v>
+        <v>51</v>
       </c>
       <c r="B106">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="B107">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>36</v>
+        <v>53</v>
       </c>
       <c r="B108">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="B109">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="B110">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="B111">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="B112">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>41</v>
-      </c>
-      <c r="B113" s="1">
-        <v>1</v>
+        <v>50</v>
+      </c>
+      <c r="B113">
+        <v>6</v>
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="B114">
         <v>1</v>
@@ -1506,207 +1559,207 @@
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="B115">
-        <v>19</v>
+        <v>5</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="B116">
-        <v>19</v>
+        <v>5</v>
       </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="B117">
-        <v>19</v>
+        <v>5</v>
       </c>
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="B118">
-        <v>20</v>
+        <v>5</v>
       </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="B119">
-        <v>20</v>
+        <v>5</v>
       </c>
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="B120">
-        <v>20</v>
+        <v>5</v>
       </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="B121">
-        <v>20</v>
+        <v>5</v>
       </c>
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="B122">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B123">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="B124">
-        <v>20</v>
+        <v>5</v>
       </c>
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="B125">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="B126">
-        <v>20</v>
+        <v>5</v>
       </c>
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="B127">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="B128">
-        <v>20</v>
+        <v>3</v>
       </c>
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="B129">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="B130">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="131" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="B131">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="B132">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="B133">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="B134">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="B135">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>40</v>
+        <v>62</v>
       </c>
       <c r="B136">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="B137">
-        <v>19</v>
+        <v>3</v>
       </c>
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="B138">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B139">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="140" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>48</v>
+        <v>63</v>
       </c>
       <c r="B140">
         <v>1</v>
@@ -1714,15 +1767,15 @@
     </row>
     <row r="141" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>47</v>
+        <v>64</v>
       </c>
       <c r="B141">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>48</v>
+        <v>64</v>
       </c>
       <c r="B142">
         <v>3</v>
@@ -1730,7 +1783,7 @@
     </row>
     <row r="143" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="B143">
         <v>1</v>
@@ -1738,7 +1791,7 @@
     </row>
     <row r="144" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="B144">
         <v>3</v>
@@ -1746,39 +1799,39 @@
     </row>
     <row r="145" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>36</v>
+        <v>66</v>
       </c>
       <c r="B145">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="146" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>36</v>
+        <v>66</v>
       </c>
       <c r="B146">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="147" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>48</v>
+        <v>67</v>
       </c>
       <c r="B147">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="148" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>47</v>
+        <v>67</v>
       </c>
       <c r="B148">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="149" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="B149">
         <v>1</v>
@@ -1786,31 +1839,31 @@
     </row>
     <row r="150" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>51</v>
+        <v>68</v>
       </c>
       <c r="B150">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="151" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="B151">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="152" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="B152">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="153" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="B153">
         <v>1</v>
@@ -1818,382 +1871,678 @@
     </row>
     <row r="154" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="B154">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="155" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="B155">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="156" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>51</v>
+        <v>71</v>
       </c>
       <c r="B156">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="157" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>50</v>
+        <v>72</v>
       </c>
       <c r="B157">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="158" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="B158">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="159" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>23</v>
+        <v>73</v>
       </c>
       <c r="B159">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="160" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>24</v>
+        <v>74</v>
       </c>
       <c r="B160">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="161" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>25</v>
+        <v>75</v>
       </c>
       <c r="B161">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="162" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>26</v>
+        <v>76</v>
       </c>
       <c r="B162">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="163" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="B163">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="164" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="B164">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="165" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="B165">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="166" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="B166">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="167" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>49</v>
+        <v>5</v>
       </c>
       <c r="B167">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="168" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="B168">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="169" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>51</v>
+        <v>7</v>
       </c>
       <c r="B169">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="170" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>53</v>
+        <v>8</v>
       </c>
       <c r="B170">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="171" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>54</v>
+        <v>9</v>
       </c>
       <c r="B171">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="172" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>54</v>
+        <v>10</v>
       </c>
       <c r="B172">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="173" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>52</v>
+        <v>11</v>
       </c>
       <c r="B173">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="174" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>56</v>
+        <v>12</v>
       </c>
       <c r="B174">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="175" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>57</v>
+        <v>13</v>
       </c>
       <c r="B175">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="176" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>58</v>
+        <v>14</v>
       </c>
       <c r="B176">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="177" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>59</v>
+        <v>15</v>
       </c>
       <c r="B177">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="178" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>60</v>
+        <v>16</v>
       </c>
       <c r="B178">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="179" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>61</v>
+        <v>17</v>
       </c>
       <c r="B179">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="180" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>62</v>
+        <v>18</v>
       </c>
       <c r="B180">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="181" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>62</v>
+        <v>19</v>
       </c>
       <c r="B181">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="182" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>62</v>
+        <v>20</v>
       </c>
       <c r="B182">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="183" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>53</v>
+        <v>21</v>
       </c>
       <c r="B183">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="184" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>63</v>
+        <v>22</v>
       </c>
       <c r="B184">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="185" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>64</v>
+        <v>23</v>
       </c>
       <c r="B185">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="186" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>64</v>
+        <v>24</v>
       </c>
       <c r="B186">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="187" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>65</v>
+        <v>25</v>
       </c>
       <c r="B187">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="188" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>65</v>
+        <v>26</v>
       </c>
       <c r="B188">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="189" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>66</v>
+        <v>27</v>
       </c>
       <c r="B189">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="190" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>66</v>
+        <v>28</v>
       </c>
       <c r="B190">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="191" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>67</v>
+        <v>29</v>
       </c>
       <c r="B191">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="192" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>67</v>
+        <v>30</v>
       </c>
       <c r="B192">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="193" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>68</v>
+        <v>31</v>
       </c>
       <c r="B193">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="194" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>68</v>
+        <v>32</v>
       </c>
       <c r="B194">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="195" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>69</v>
+        <v>33</v>
       </c>
       <c r="B195">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="196" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>69</v>
+        <v>34</v>
       </c>
       <c r="B196">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="197" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="B197">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="198" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>70</v>
+        <v>36</v>
       </c>
       <c r="B198">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="199" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>71</v>
+        <v>37</v>
       </c>
       <c r="B199">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="200" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
+        <v>38</v>
+      </c>
+      <c r="B200">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A201" t="s">
+        <v>39</v>
+      </c>
+      <c r="B201">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A202" t="s">
+        <v>40</v>
+      </c>
+      <c r="B202">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A203" t="s">
+        <v>41</v>
+      </c>
+      <c r="B203">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A204" t="s">
+        <v>42</v>
+      </c>
+      <c r="B204">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A205" t="s">
+        <v>43</v>
+      </c>
+      <c r="B205">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A206" t="s">
+        <v>44</v>
+      </c>
+      <c r="B206">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A207" t="s">
+        <v>45</v>
+      </c>
+      <c r="B207">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A208" t="s">
+        <v>46</v>
+      </c>
+      <c r="B208">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A209" t="s">
+        <v>52</v>
+      </c>
+      <c r="B209">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="210" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A210" t="s">
+        <v>47</v>
+      </c>
+      <c r="B210">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="211" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A211" t="s">
+        <v>48</v>
+      </c>
+      <c r="B211">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="212" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A212" t="s">
+        <v>49</v>
+      </c>
+      <c r="B212">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A213" t="s">
+        <v>50</v>
+      </c>
+      <c r="B213">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A214" t="s">
+        <v>51</v>
+      </c>
+      <c r="B214">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="215" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A215" t="s">
+        <v>53</v>
+      </c>
+      <c r="B215">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A216" t="s">
+        <v>54</v>
+      </c>
+      <c r="B216">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="217" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A217" t="s">
+        <v>55</v>
+      </c>
+      <c r="B217">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="218" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A218" t="s">
+        <v>52</v>
+      </c>
+      <c r="B218">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="219" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A219" t="s">
+        <v>56</v>
+      </c>
+      <c r="B219">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="220" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A220" t="s">
+        <v>57</v>
+      </c>
+      <c r="B220">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="221" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A221" t="s">
+        <v>58</v>
+      </c>
+      <c r="B221">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="222" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A222" t="s">
+        <v>59</v>
+      </c>
+      <c r="B222">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="223" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A223" t="s">
+        <v>60</v>
+      </c>
+      <c r="B223">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="224" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A224" t="s">
+        <v>61</v>
+      </c>
+      <c r="B224">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="225" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A225" t="s">
+        <v>62</v>
+      </c>
+      <c r="B225">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="226" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A226" t="s">
+        <v>63</v>
+      </c>
+      <c r="B226">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="227" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A227" t="s">
+        <v>64</v>
+      </c>
+      <c r="B227">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="228" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A228" t="s">
+        <v>65</v>
+      </c>
+      <c r="B228">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="229" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A229" t="s">
+        <v>66</v>
+      </c>
+      <c r="B229">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="230" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A230" t="s">
+        <v>67</v>
+      </c>
+      <c r="B230">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="231" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A231" t="s">
+        <v>68</v>
+      </c>
+      <c r="B231">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="232" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A232" t="s">
+        <v>69</v>
+      </c>
+      <c r="B232">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="233" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A233" t="s">
+        <v>70</v>
+      </c>
+      <c r="B233">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="234" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A234" t="s">
         <v>71</v>
       </c>
-      <c r="B200">
-        <v>3</v>
+      <c r="B234">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="235" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A235" t="s">
+        <v>72</v>
+      </c>
+      <c r="B235">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="236" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A236" t="s">
+        <v>73</v>
+      </c>
+      <c r="B236">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="237" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A237" t="s">
+        <v>74</v>
+      </c>
+      <c r="B237">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B171" xr:uid="{582B0F33-0746-4ED0-86AD-A10E2401FD21}"/>
+  <autoFilter ref="A1:B237" xr:uid="{582B0F33-0746-4ED0-86AD-A10E2401FD21}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>